<commit_message>
added requery before retrieval
</commit_message>
<xml_diff>
--- a/tests/results/eval-log.xlsx
+++ b/tests/results/eval-log.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="49">
   <si>
     <t>Date</t>
   </si>
@@ -67,6 +67,21 @@
     <t>Avg Chunk Count</t>
   </si>
   <si>
+    <t>Answer Quality Pass Rate</t>
+  </si>
+  <si>
+    <t>Conversation Condensation Accuracy</t>
+  </si>
+  <si>
+    <t>Conversation Retrieval Recall</t>
+  </si>
+  <si>
+    <t>Decomposition Coverage (Triggered)</t>
+  </si>
+  <si>
+    <t>Decomposition Coverage (All Docs)</t>
+  </si>
+  <si>
     <t>2026-08-12T11:54:46.293Z</t>
   </si>
   <si>
@@ -113,6 +128,36 @@
   </si>
   <si>
     <t>dynamic-k, threshold=0.65, maxK=8</t>
+  </si>
+  <si>
+    <t>2026-08-13T05:09:30.479Z</t>
+  </si>
+  <si>
+    <t>tests\results\eval-2026-08-13T05-09-30-478Z.json</t>
+  </si>
+  <si>
+    <t>dynamic-k, threshold=0.60, maxK=8</t>
+  </si>
+  <si>
+    <t>2026-08-13T08:48:03.378Z</t>
+  </si>
+  <si>
+    <t>tests\results\eval-2026-08-13T08-48-03-371Z.json</t>
+  </si>
+  <si>
+    <t>baseline single-turn, phase 1</t>
+  </si>
+  <si>
+    <t>2026-08-13T09:09:51.844Z</t>
+  </si>
+  <si>
+    <t>tests\results\eval-2026-08-13T09-09-51-839Z.json</t>
+  </si>
+  <si>
+    <t>phase3 conversations test</t>
+  </si>
+  <si>
+    <t>3/5</t>
   </si>
 </sst>
 </file>
@@ -493,13 +538,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R6"/>
+  <dimension ref="A1:W9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="18" width="20" customWidth="1"/>
+    <col min="1" max="23" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -553,11 +598,26 @@
       </c>
       <c r="R1" s="1" t="s">
         <v>17</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="B2">
         <v>60</v>
@@ -593,15 +653,15 @@
         <v>0</v>
       </c>
       <c r="M2" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="N2" t="s">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B3">
         <v>60</v>
@@ -637,15 +697,15 @@
         <v>0</v>
       </c>
       <c r="M3" t="s">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="N3" t="s">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="B4">
         <v>60</v>
@@ -681,18 +741,18 @@
         <v>0</v>
       </c>
       <c r="M4" t="s">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="N4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="O4" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B5">
         <v>65</v>
@@ -728,13 +788,13 @@
         <v>0</v>
       </c>
       <c r="M5" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="N5" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="O5" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="P5">
         <v>1</v>
@@ -748,7 +808,7 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B6">
         <v>65</v>
@@ -784,13 +844,13 @@
         <v>0</v>
       </c>
       <c r="M6" t="s">
+        <v>37</v>
+      </c>
+      <c r="N6" t="s">
+        <v>38</v>
+      </c>
+      <c r="O6" t="s">
         <v>32</v>
-      </c>
-      <c r="N6" t="s">
-        <v>33</v>
-      </c>
-      <c r="O6" t="s">
-        <v>27</v>
       </c>
       <c r="P6">
         <v>0.4</v>
@@ -800,6 +860,192 @@
       </c>
       <c r="R6">
         <v>1.662</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>39</v>
+      </c>
+      <c r="B7">
+        <v>65</v>
+      </c>
+      <c r="C7">
+        <v>20</v>
+      </c>
+      <c r="D7">
+        <v>0.969</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7">
+        <v>1</v>
+      </c>
+      <c r="H7">
+        <v>0.985</v>
+      </c>
+      <c r="I7">
+        <v>0.984</v>
+      </c>
+      <c r="J7">
+        <v>0.923</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7" t="s">
+        <v>40</v>
+      </c>
+      <c r="N7" t="s">
+        <v>41</v>
+      </c>
+      <c r="O7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P7">
+        <v>0.8</v>
+      </c>
+      <c r="Q7">
+        <v>0.833</v>
+      </c>
+      <c r="R7">
+        <v>1.944</v>
+      </c>
+    </row>
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B8">
+        <v>65</v>
+      </c>
+      <c r="C8">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>0.969</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
+        <v>1</v>
+      </c>
+      <c r="H8">
+        <v>0.985</v>
+      </c>
+      <c r="I8">
+        <v>0.984</v>
+      </c>
+      <c r="J8">
+        <v>0.923</v>
+      </c>
+      <c r="K8">
+        <v>1</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8" t="s">
+        <v>43</v>
+      </c>
+      <c r="N8" t="s">
+        <v>44</v>
+      </c>
+      <c r="O8" t="s">
+        <v>32</v>
+      </c>
+      <c r="P8">
+        <v>0.8</v>
+      </c>
+      <c r="Q8">
+        <v>0.833</v>
+      </c>
+      <c r="R8">
+        <v>1.944</v>
+      </c>
+      <c r="S8">
+        <v>0.972</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B9">
+        <v>65</v>
+      </c>
+      <c r="C9">
+        <v>20</v>
+      </c>
+      <c r="D9">
+        <v>0.862</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9">
+        <v>1</v>
+      </c>
+      <c r="H9">
+        <v>0.923</v>
+      </c>
+      <c r="I9">
+        <v>0.94</v>
+      </c>
+      <c r="J9">
+        <v>0.692</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9" t="s">
+        <v>46</v>
+      </c>
+      <c r="N9" t="s">
+        <v>47</v>
+      </c>
+      <c r="O9" t="s">
+        <v>1</v>
+      </c>
+      <c r="P9">
+        <v>1</v>
+      </c>
+      <c r="Q9">
+        <v>0</v>
+      </c>
+      <c r="R9">
+        <v>8</v>
+      </c>
+      <c r="S9" t="s">
+        <v>28</v>
+      </c>
+      <c r="T9">
+        <v>0.6</v>
+      </c>
+      <c r="U9">
+        <v>1</v>
+      </c>
+      <c r="V9" t="s">
+        <v>48</v>
+      </c>
+      <c r="W9" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>